<commit_message>
Added thin border & initial warning msg
</commit_message>
<xml_diff>
--- a/weekly_goals.xlsx
+++ b/weekly_goals.xlsx
@@ -53,7 +53,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="6">
+  <borders count="10">
     <border>
       <left/>
       <right/>
@@ -77,52 +77,100 @@
       <diagonal/>
     </border>
     <border>
-      <left style="thick"/>
-      <right style="thick"/>
-      <top style="thick"/>
-      <bottom style="thick"/>
-    </border>
-    <border>
-      <left style="thick"/>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
       <right/>
       <top/>
       <bottom/>
       <diagonal/>
     </border>
     <border>
-      <left style="thick"/>
-      <right style="thick"/>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
       <top/>
       <bottom/>
       <diagonal/>
     </border>
     <border>
-      <left style="thick"/>
-      <right style="thick"/>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
       <top/>
-      <bottom style="thick"/>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
       <diagonal/>
+    </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom/>
+    </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top/>
+      <bottom/>
+    </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top/>
+      <bottom style="thin"/>
     </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -488,198 +536,151 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C13"/>
+  <dimension ref="A2:D21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
-    <col width="12.109375" customWidth="1" style="3" min="1" max="1"/>
-    <col width="24.6640625" customWidth="1" style="3" min="2" max="2"/>
-    <col width="15.6640625" customWidth="1" style="3" min="3" max="3"/>
+    <col width="24.77734375" customWidth="1" style="4" min="3" max="3"/>
+    <col width="14.5546875" customWidth="1" style="4" min="4" max="4"/>
   </cols>
   <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+    <row r="2">
+      <c r="B2" s="1" t="inlineStr">
         <is>
           <t>Week</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="C2" s="1" t="inlineStr">
         <is>
           <t>Goal</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="D2" s="1" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" s="2" t="inlineStr">
-        <is>
-          <t>Week 3</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
+    <row r="4">
+      <c r="B4" s="5" t="n"/>
+      <c r="C4" s="3" t="inlineStr">
         <is>
           <t>Learn Docker basics</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>✅ Done</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="B3" t="inlineStr">
+      <c r="D4" s="3" t="n"/>
+    </row>
+    <row r="5">
+      <c r="C5" s="3" t="inlineStr">
         <is>
           <t>Complete internship task</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>❌ Not Done</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="B4" t="inlineStr">
+      <c r="D5" s="3" t="n"/>
+    </row>
+    <row r="6">
+      <c r="C6" s="3" t="inlineStr">
         <is>
           <t>Read 15 pages</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>✅ Done</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="B5" t="inlineStr">
+      <c r="D6" s="3" t="n"/>
+    </row>
+    <row r="7">
+      <c r="C7" s="3" t="inlineStr">
         <is>
           <t>Review Angular signals</t>
         </is>
       </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>✅ Done</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="4" t="inlineStr">
-        <is>
-          <t>Week 3</t>
-        </is>
-      </c>
-      <c r="B6" s="5" t="inlineStr">
+      <c r="D7" s="3" t="n"/>
+    </row>
+    <row r="9">
+      <c r="B9" s="5" t="n"/>
+      <c r="C9" s="3" t="inlineStr">
         <is>
           <t>Learn Docker basics</t>
         </is>
       </c>
-      <c r="C6" s="5" t="inlineStr">
-        <is>
-          <t>✅ Done</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="6" t="n"/>
-      <c r="B7" s="5" t="inlineStr">
+      <c r="D9" s="3" t="n"/>
+    </row>
+    <row r="10">
+      <c r="B10" s="6" t="n"/>
+      <c r="C10" s="3" t="inlineStr">
         <is>
           <t>Complete internship task</t>
         </is>
       </c>
-      <c r="C7" s="5" t="inlineStr">
-        <is>
-          <t>❌ Not Done</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="6" t="n"/>
-      <c r="B8" s="5" t="inlineStr">
+      <c r="D10" s="3" t="n"/>
+    </row>
+    <row r="11">
+      <c r="B11" s="6" t="n"/>
+      <c r="C11" s="3" t="inlineStr">
         <is>
           <t>Read 15 pages</t>
         </is>
       </c>
-      <c r="C8" s="5" t="inlineStr">
-        <is>
-          <t>✅ Done</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="7" t="n"/>
-      <c r="B9" s="5" t="inlineStr">
+      <c r="D11" s="3" t="n"/>
+    </row>
+    <row r="12">
+      <c r="B12" s="7" t="n"/>
+      <c r="C12" s="3" t="inlineStr">
         <is>
           <t>Review Angular signals</t>
         </is>
       </c>
-      <c r="C9" s="5" t="inlineStr">
-        <is>
-          <t>✅ Done</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="8" t="inlineStr">
-        <is>
-          <t>Week 3</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
+      <c r="D12" s="3" t="n"/>
+    </row>
+    <row r="16">
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>        </t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="B18" s="8" t="inlineStr">
+        <is>
+          <t>Apr 13 - Apr 19</t>
+        </is>
+      </c>
+      <c r="C18" s="9" t="inlineStr">
         <is>
           <t>Learn Docker basics</t>
         </is>
       </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>✅ Done</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="B11" t="inlineStr">
+      <c r="D18" s="9" t="inlineStr"/>
+    </row>
+    <row r="19">
+      <c r="B19" s="10" t="n"/>
+      <c r="C19" s="9" t="inlineStr">
         <is>
           <t>Complete internship task</t>
         </is>
       </c>
-      <c r="C11" t="inlineStr">
-        <is>
-          <t>❌ Not Done</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="B12" t="inlineStr">
+      <c r="D19" s="9" t="inlineStr"/>
+    </row>
+    <row r="20">
+      <c r="B20" s="10" t="n"/>
+      <c r="C20" s="9" t="inlineStr">
         <is>
           <t>Read 15 pages</t>
         </is>
       </c>
-      <c r="C12" t="inlineStr">
-        <is>
-          <t>✅ Done</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="B13" t="inlineStr">
+      <c r="D20" s="9" t="inlineStr"/>
+    </row>
+    <row r="21">
+      <c r="B21" s="11" t="n"/>
+      <c r="C21" s="9" t="inlineStr">
         <is>
           <t>Review Angular signals</t>
         </is>
       </c>
-      <c r="C13" t="inlineStr">
-        <is>
-          <t>✅ Done</t>
-        </is>
-      </c>
+      <c r="D21" s="9" t="inlineStr"/>
     </row>
   </sheetData>
   <mergeCells count="3">
-    <mergeCell ref="A2:A5"/>
-    <mergeCell ref="A10:A13"/>
-    <mergeCell ref="A6:A9"/>
+    <mergeCell ref="A4:A7"/>
+    <mergeCell ref="B18:B21"/>
+    <mergeCell ref="B9:B12"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>